<commit_message>
fix(documents): 통관SET 날짜 serial(43705) 버그 + 말소증 등록번호칸 2줄 분리
날짜 버그: applyCurrency 가 통화 적응 시 '$'를 전부 통화기호로 바꿔
영문 날짜서식 로케일 토큰 [$-409] 까지 깨뜨림 → 비-USD(EUR 등) 차량은
[€-409] 가 되어 Excel 이 서식을 못 읽고 등록증날짜를 serial(43705)로 표시.
preg_replace('/\$(?!-)/') 로 변경 — 로케일 '$'(뒤가 '-')는 보존, 금액 '$'만 변환.
영문등록증(O3·L13)·컨테이너/RORO INVOICE 날짜셀 등 전 currency-aware 서류 일괄 해결.

말소증: 라벨이 자동차등록번호/Registration No. 2줄인데 값칸 E8:G9 가 1줄 병합이라
차량번호만 표시. E8:G8(=구매리스트!B4 차량번호) / E9:G9(=구매리스트!D4 영문차량번호)
2줄로 분리. system/heyman/karaba 3개 세트 모두 적용(scripts/split-malso-plate-cells.php).

회귀 테스트 추가(EUR 통관 날짜 로케일 보존) + 통화 테스트 헬퍼 정합.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/clearance_set.xlsx
+++ b/resources/templates/heyman/clearance_set.xlsx
@@ -10063,8 +10063,12 @@
         </is>
       </c>
       <c r="D9" s="304"/>
-      <c r="E9" s="305"/>
-      <c r="G9" s="304"/>
+      <c r="E9" s="184" t="str">
+        <f>구매리스트!D4</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="184"/>
+      <c r="G9" s="184"/>
       <c r="H9" s="180" t="inlineStr">
         <is>
           <r>
@@ -11130,7 +11134,6 @@
     <mergeCell ref="H22:J22"/>
     <mergeCell ref="H19:J19"/>
     <mergeCell ref="A5:O5"/>
-    <mergeCell ref="E8:G9"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="K33:N33"/>
     <mergeCell ref="A49:J49"/>
@@ -11208,6 +11211,8 @@
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="H25:J25"/>
     <mergeCell ref="G34:K34"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E9:G9"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true" horizontalCentered="true"/>
   <pageMargins left="0.31496062992126" right="0.23622047244094" top="0.45" bottom="0.51181102362205" header="0.31496062992126" footer="0.31496062992126"/>

</xml_diff>

<commit_message>
fix(documents): 계약서 Bank/Beneficiary 주소 분리 + 차량인보이스·팩킹 발행일 TODAY
- 컨테이너/RORO 계약서(heyman): F12:G13 병합 분리 → F12=Bank Adress / F13=Beneficiary Adress(heyman 주소).
  병합 때문에 수취인 주소 칸이 없어 빈칸이던 것 해소.
- 통관SET 차량인보이스·차량팩킹 I11(8. date of invoice): =구매리스트!D11(선적일) → =TODAY()(발행일).
  D11은 C18 선적일 cascade에 계속 사용되어 무관.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/clearance_set.xlsx
+++ b/resources/templates/heyman/clearance_set.xlsx
@@ -3516,7 +3516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="402">
+  <cellXfs count="401">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
@@ -4719,9 +4719,6 @@
     </xf>
     <xf xfId="0" fontId="11" numFmtId="0" fillId="0" borderId="56" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9030,7 +9027,7 @@
           </r>
         </is>
       </c>
-      <c r="I23" s="401" t="str">
+      <c r="I23" s="11" t="str">
         <f>구매리스트!I9</f>
         <v>0</v>
       </c>
@@ -11434,7 +11431,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="53" t="str">
-        <f>구매리스트!D11</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
     </row>
@@ -12452,7 +12449,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="53" t="str">
-        <f>구매리스트!D11</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(documents): 계약서 Bank/Beneficiary 주소 분리 + 인보이스 발행일 TODAY + 브랜드 라벨
- 컨테이너/RORO 계약서(heyman): F12:G13 병합 분리 → Bank Adress(F12)/Beneficiary Adress(F13=heyman)
- 통관SET 차량인보이스·차량팩킹 I11: 선적일 → =TODAY()(발행일)
- 기본정보 brand 라벨 '제조사'→'브랜드' (NICE 제원 '제조사'와 혼동 해소)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/clearance_set.xlsx
+++ b/resources/templates/heyman/clearance_set.xlsx
@@ -3516,7 +3516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="402">
+  <cellXfs count="401">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
@@ -4719,9 +4719,6 @@
     </xf>
     <xf xfId="0" fontId="11" numFmtId="0" fillId="0" borderId="56" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9030,7 +9027,7 @@
           </r>
         </is>
       </c>
-      <c r="I23" s="401" t="str">
+      <c r="I23" s="11" t="str">
         <f>구매리스트!I9</f>
         <v>0</v>
       </c>
@@ -11434,7 +11431,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="53" t="str">
-        <f>구매리스트!D11</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
     </row>
@@ -12452,7 +12449,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="53" t="str">
-        <f>구매리스트!D11</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(documents): 선적 인보이스 Vessel name 보완 + 통관SET 정부직인 교체
- 컨테이너/RORO 인보이스&팩킹: Vessel name(B18) 매핑 누락 보완
- 통관SET 한글/영문등록증·말소증 정부직인(구 시흥시장 인장) 신규 직인으로 교체

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/clearance_set.xlsx
+++ b/resources/templates/heyman/clearance_set.xlsx
@@ -4741,22 +4741,17 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>14</xdr:col>
       <xdr:colOff>600075</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="1057275" cy="1028700"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="그림 32" descr=""/>
+        <xdr:cNvPr id="2" name="govt_seal" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4768,16 +4763,14 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:ext cx="1057275" cy="1028700"/>
-        </a:xfrm>
+        <a:xfrm rot="0"/>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4822,43 +4815,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>638175</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>457200</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="그림 4" descr=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:ext cx="1057275" cy="1028700"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>28575</xdr:colOff>
       <xdr:row>11</xdr:row>
@@ -4872,13 +4828,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="그림 12" descr=""/>
+        <xdr:cNvPr id="2" name="그림 12" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4894,6 +4850,36 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>638175</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1057275" cy="1028700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="govt_seal" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="0"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4938,43 +4924,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>447675</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="그림 4" descr=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:ext cx="1247775" cy="1228725"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
       <xdr:row>48</xdr:row>
@@ -4988,13 +4937,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="그림 7" descr=""/>
+        <xdr:cNvPr id="2" name="그림 7" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5010,6 +4959,36 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>447675</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1247775" cy="1228725"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="govt_seal" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="0"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>

<commit_message>
fix(documents): 서류 4건 — 통관 RORO 표기·말소 FOB 인코텀즈·HEYMAN TEL/FAX
코드(전 세트):
- 통관SET 구매리스트 B12: RORO 면 'RORO'(차량인보이스 G2/G3 cascade 표기),
  아니면 컨테이너번호 — 로로 시 참조셀 빈칸 방지.
- 말소계약서 D50: 'F.O.B INCHOEN PORT' 의 FOB 를 수출통관 탭 incoterms(FOB/CFR)에서.
  미입력 시 'F.O.B' 유지.

HEYMAN 템플릿(정적 셀):
- 말소계약서 E5 FAX: SSANCAR 거(82-031-499-1989) → HEYMAN 82-505-366-9977.
- 컨/RORO 인보이스 INVOICE B3 + 통관 차량인보이스/팩킹 A3 TEL → 82-10-9009-9977
  (TEL: 프리픽스로 한정 치환, FAX 보존). RichText 런 in-place 수정으로 brandHeader 호환.

테스트 5: D50 incoterms/fallback·B12 RORO cascade/컨테이너·HEYMAN 재저장 무결성
(clearance 크로스시트 수식 생존). 전 스위트 755 통과.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/clearance_set.xlsx
+++ b/resources/templates/heyman/clearance_set.xlsx
@@ -1591,7 +1591,7 @@
     <r>
       <t xml:space="preserve">SSANCAR LTD.,
 #513, THE PARK 365, 50 Seonyudong1-ro, Yeongdeungpo-gu, Seoul, Korea
-TEL:82-505-366-9977 
+TEL:82-10-9009-9977 
 FAX:82-505-366-9977
 EMAIL : heyman99888@gmail.com</t>
     </r>
@@ -1774,7 +1774,7 @@
   <si>
     <t>HEYMAN LTD.,
 #513, THE PARK 365, 50 Seonyudong1-ro, Yeongdeungpo-gu, Seoul, Korea
-TEL:82-505-366-9977 
+TEL:82-10-9009-9977 
 FAX:82-505-366-9977
 EMAIL : heyman99888@gmail.com</t>
   </si>
@@ -4704,6 +4704,36 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1057275" cy="1028700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="govt_seal" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="0"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -4719,13 +4749,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="그림 30" descr=""/>
+        <xdr:cNvPr id="2" name="그림 30" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4741,23 +4771,28 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
+      <xdr:colOff>638175</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1057275" cy="1028700"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="govt_seal" descr=""/>
+        <xdr:cNvPr id="1" name="govt_seal" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4771,11 +4806,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -4791,13 +4821,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="그림 3" descr=""/>
+        <xdr:cNvPr id="2" name="그림 3" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4828,13 +4858,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="그림 12" descr=""/>
+        <xdr:cNvPr id="3" name="그림 12" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4850,23 +4880,28 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>638175</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>447675</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1057275" cy="1028700"/>
+    <xdr:ext cx="1247775" cy="1228725"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="govt_seal" descr=""/>
+        <xdr:cNvPr id="1" name="govt_seal" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4880,11 +4915,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -4900,13 +4930,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="그림 2" descr=""/>
+        <xdr:cNvPr id="2" name="그림 2" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4937,13 +4967,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="그림 7" descr=""/>
+        <xdr:cNvPr id="3" name="그림 7" descr=""/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4959,36 +4989,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>447675</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1247775" cy="1228725"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="govt_seal" descr=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="0"/>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -11245,7 +11245,7 @@
           <r>
             <t xml:space="preserve">SSANCAR LTD.,
 #513, THE PARK 365, 50 Seonyudong1-ro, Yeongdeungpo-gu, Seoul, Korea
-TEL:82-505-366-9977 
+TEL:82-10-9009-9977 
 FAX:82-505-366-9977
 EMAIL : heyman99888@gmail.com</t>
           </r>

</xml_diff>